<commit_message>
Update scoreboard and monitor
</commit_message>
<xml_diff>
--- a/Vplan_8bit_timer.xlsx
+++ b/Vplan_8bit_timer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Quang Tran\Projects\project1\ICTC-APB-8bit-Timer-Verification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AD48AE-D187-495C-B64C-0630E48C937E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE4E075-C44D-43B2-95EC-FBF223E27EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1200,7 +1200,7 @@
         <v>24</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>175</v>
+        <v>25</v>
       </c>
       <c r="I11" s="7"/>
       <c r="J11" s="8"/>

</xml_diff>